<commit_message>
catgeory bulk upload process
</commit_message>
<xml_diff>
--- a/public/uploads/files/SampleFormatCategoryValues.xlsx
+++ b/public/uploads/files/SampleFormatCategoryValues.xlsx
@@ -27,30 +27,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="8">
   <si>
-    <t>CategoryName</t>
+    <t>ParentName</t>
   </si>
   <si>
-    <t>ParentId</t>
+    <t>SubCatgoryName</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>ShowOnHome</t>
+    <t>none</t>
   </si>
   <si>
-    <t>samplecheck</t>
-  </si>
-  <si>
-    <t>none</t>
+    <t>Geocery</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
-    <t>No</t>
+    <t>Refrigerator</t>
+  </si>
+  <si>
+    <t>Item1</t>
   </si>
 </sst>
 </file>
@@ -1056,10 +1056,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelRow="1" outlineLevelCol="3"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelCol="2"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1069,22 +1069,104 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
         <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bulk category upload process
</commit_message>
<xml_diff>
--- a/public/uploads/files/SampleFormatCategoryValues.xlsx
+++ b/public/uploads/files/SampleFormatCategoryValues.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="19890" windowHeight="4485"/>
+    <workbookView windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>ParentName</t>
   </si>
@@ -47,10 +47,16 @@
     <t>Active</t>
   </si>
   <si>
-    <t>Refrigerator</t>
+    <t>Item1</t>
   </si>
   <si>
-    <t>Item1</t>
+    <t>Gadgets</t>
+  </si>
+  <si>
+    <t>Gadgets&gt;Item1</t>
+  </si>
+  <si>
+    <t>Item2</t>
   </si>
 </sst>
 </file>
@@ -63,13 +69,19 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -526,153 +538,155 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1056,8 +1070,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="41" customWidth="1"/>
+    <col min="2" max="2" width="34.125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -1083,91 +1101,42 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="4" s="1" customFormat="1" spans="1:3">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="5" s="1" customFormat="1" spans="1:3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
+    <row r="11" ht="18" spans="1:1">
+      <c r="A11" s="2"/>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
+    <row r="12" ht="18" spans="1:1">
+      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
sample category bulk upload file
</commit_message>
<xml_diff>
--- a/public/uploads/files/SampleFormatCategoryValues.xlsx
+++ b/public/uploads/files/SampleFormatCategoryValues.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
   <si>
     <t>ParentName</t>
   </si>
@@ -41,22 +41,31 @@
     <t>none</t>
   </si>
   <si>
-    <t>Geocery</t>
+    <t>Large Appliance</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
-    <t>Item1</t>
+    <t>Air Conditioner</t>
+  </si>
+  <si>
+    <t>Large Appliance&gt;Air Conditioner</t>
+  </si>
+  <si>
+    <t>Cassette AC</t>
   </si>
   <si>
     <t>Gadgets</t>
   </si>
   <si>
-    <t>Gadgets&gt;Item1</t>
-  </si>
-  <si>
-    <t>Item2</t>
+    <t>Smart Watches</t>
+  </si>
+  <si>
+    <t>Gadgets&gt;Smart Watches</t>
+  </si>
+  <si>
+    <t>NewRoundedWatches</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1124,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>5</v>
@@ -1123,12 +1132,34 @@
     </row>
     <row r="5" s="1" customFormat="1" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>